<commit_message>
fix: make UEQ golden fixture discriminative
</commit_message>
<xml_diff>
--- a/docs/research/ueq-saw-golden-fixture.xlsx
+++ b/docs/research/ueq-saw-golden-fixture.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra1e3448186b34346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Mapping" sheetId="2" r:id="Rb34b6f7fdcea449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Answers" sheetId="3" r:id="Rbfb99a8e038b4683"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformed Scores" sheetId="4" r:id="R2f50706ff0c141c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respondent Scale Means" sheetId="5" r:id="R50d7b2e53d604f36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical and SAW" sheetId="6" r:id="R64a112157ed64b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd468ca3291f7411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Mapping" sheetId="2" r:id="R1aade2b990974955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Answers" sheetId="3" r:id="Re9e1450f95aa43c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformed Scores" sheetId="4" r:id="Rba32031370714ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respondent Scale Means" sheetId="5" r:id="R96dbf4eac15f4c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical and SAW" sheetId="6" r:id="R12621751a14f430e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -385,6 +385,7 @@
     <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -399,6 +400,7 @@
       <x:c r="G1" s="3"/>
       <x:c r="H1" s="3"/>
       <x:c r="I1" s="3"/>
+      <x:c r="J1" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -413,7 +415,8 @@
       <x:c r="F3" s="23"/>
       <x:c r="G3" s="23"/>
       <x:c r="H3" s="23"/>
-      <x:c r="I3" s="24"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="24"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
@@ -428,7 +431,8 @@
       <x:c r="F4" s="12"/>
       <x:c r="G4" s="12"/>
       <x:c r="H4" s="12"/>
-      <x:c r="I4" s="13"/>
+      <x:c r="I4" s="12"/>
+      <x:c r="J4" s="13"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
@@ -443,7 +447,8 @@
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="12"/>
       <x:c r="H5" s="12"/>
-      <x:c r="I5" s="13"/>
+      <x:c r="I5" s="12"/>
+      <x:c r="J5" s="13"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="str">
@@ -458,7 +463,8 @@
       <x:c r="F6" s="12"/>
       <x:c r="G6" s="12"/>
       <x:c r="H6" s="12"/>
-      <x:c r="I6" s="13"/>
+      <x:c r="I6" s="12"/>
+      <x:c r="J6" s="13"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="11" t="str">
@@ -473,7 +479,8 @@
       <x:c r="F7" s="12"/>
       <x:c r="G7" s="12"/>
       <x:c r="H7" s="12"/>
-      <x:c r="I7" s="13"/>
+      <x:c r="I7" s="12"/>
+      <x:c r="J7" s="13"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="11" t="str">
@@ -488,7 +495,8 @@
       <x:c r="F8" s="12"/>
       <x:c r="G8" s="12"/>
       <x:c r="H8" s="12"/>
-      <x:c r="I8" s="13"/>
+      <x:c r="I8" s="12"/>
+      <x:c r="J8" s="13"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="11" t="str">
@@ -503,7 +511,8 @@
       <x:c r="F9" s="12"/>
       <x:c r="G9" s="12"/>
       <x:c r="H9" s="12"/>
-      <x:c r="I9" s="13"/>
+      <x:c r="I9" s="12"/>
+      <x:c r="J9" s="13"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="11"/>
@@ -514,7 +523,8 @@
       <x:c r="F10" s="12"/>
       <x:c r="G10" s="12"/>
       <x:c r="H10" s="12"/>
-      <x:c r="I10" s="13"/>
+      <x:c r="I10" s="12"/>
+      <x:c r="J10" s="13"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11"/>
@@ -525,7 +535,8 @@
       <x:c r="F11" s="12"/>
       <x:c r="G11" s="12"/>
       <x:c r="H11" s="12"/>
-      <x:c r="I11" s="13"/>
+      <x:c r="I11" s="12"/>
+      <x:c r="J11" s="13"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="25" t="str">
@@ -538,7 +549,8 @@
       <x:c r="F12" s="22"/>
       <x:c r="G12" s="22"/>
       <x:c r="H12" s="22"/>
-      <x:c r="I12" s="26"/>
+      <x:c r="I12" s="22"/>
+      <x:c r="J12" s="26"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="27" t="str">
@@ -565,8 +577,11 @@
       <x:c r="H13" s="7" t="str">
         <x:v>CI95 upper</x:v>
       </x:c>
-      <x:c r="I13" s="28" t="str">
+      <x:c r="I13" s="7" t="str">
         <x:v>Cronbach alpha</x:v>
+      </x:c>
+      <x:c r="J13" s="28" t="str">
+        <x:v>Gap to Good</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -582,27 +597,31 @@
       </x:c>
       <x:c r="D14" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C4:F4)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E14" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C4:F4)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.5181877251716008</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:f>E14/SQRT(C14)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.2590938625858004</x:v>
       </x:c>
       <x:c r="G14" s="17" t="n">
         <x:f>D14-3.182446305284263*F14</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>-0.07455230570800908</x:v>
       </x:c>
       <x:c r="H14" s="17" t="n">
         <x:f>D14+3.182446305284263*F14</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I14" s="18" t="n">
+        <x:v>1.574552305708009</x:v>
+      </x:c>
+      <x:c r="I14" s="17" t="n">
         <x:f>(6/(6-1))*(1-(VAR.S('Transformed Scores'!D$4:D$7)+VAR.S('Transformed Scores'!O$4:O$7)+VAR.S('Transformed Scores'!Q$4:Q$7)+VAR.S('Transformed Scores'!S$4:S$7)+VAR.S('Transformed Scores'!AA$4:AA$7)+VAR.S('Transformed Scores'!AB$4:AB$7))/VAR.S('Respondent Scale Means'!G4:J4))</x:f>
-        <x:v>1</x:v>
+        <x:v>0.3517241379310345</x:v>
+      </x:c>
+      <x:c r="J14" s="18" t="n">
+        <x:f>MAX(0,$B$4-D14)</x:f>
+        <x:v>0.8300000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -618,27 +637,31 @@
       </x:c>
       <x:c r="D15" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C5:F5)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="E15" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C5:F5)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.5400617248673217</x:v>
       </x:c>
       <x:c r="F15" s="17" t="n">
         <x:f>E15/SQRT(C15)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.27003086243366087</x:v>
       </x:c>
       <x:c r="G15" s="17" t="n">
         <x:f>D15-3.182446305284263*F15</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>0.39064127953527295</x:v>
       </x:c>
       <x:c r="H15" s="17" t="n">
         <x:f>D15+3.182446305284263*F15</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I15" s="18" t="n">
+        <x:v>2.1093587204647273</x:v>
+      </x:c>
+      <x:c r="I15" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!E$4:E$7)+VAR.S('Transformed Scores'!G$4:G$7)+VAR.S('Transformed Scores'!P$4:P$7)+VAR.S('Transformed Scores'!X$4:X$7))/VAR.S('Respondent Scale Means'!G5:J5))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.2857142857142856</x:v>
+      </x:c>
+      <x:c r="J15" s="18" t="n">
+        <x:f>MAX(0,$B$5-D15)</x:f>
+        <x:v>0.48</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -658,23 +681,27 @@
       </x:c>
       <x:c r="E16" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C6:F6)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.408248290463863</x:v>
       </x:c>
       <x:c r="F16" s="17" t="n">
         <x:f>E16/SQRT(C16)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.2041241452319315</x:v>
       </x:c>
       <x:c r="G16" s="17" t="n">
         <x:f>D16-3.182446305284263*F16</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>0.3503858681873313</x:v>
       </x:c>
       <x:c r="H16" s="17" t="n">
         <x:f>D16+3.182446305284263*F16</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I16" s="18" t="n">
+        <x:v>1.6496141318126687</x:v>
+      </x:c>
+      <x:c r="I16" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!L$4:L$7)+VAR.S('Transformed Scores'!W$4:W$7)+VAR.S('Transformed Scores'!Y$4:Y$7)+VAR.S('Transformed Scores'!Z$4:Z$7))/VAR.S('Respondent Scale Means'!G6:J6))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="J16" s="18" t="n">
+        <x:f>MAX(0,$B$6-D16)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -690,27 +717,31 @@
       </x:c>
       <x:c r="D17" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C7:F7)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E17" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C7:F7)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.5400617248673217</x:v>
       </x:c>
       <x:c r="F17" s="17" t="n">
         <x:f>E17/SQRT(C17)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.27003086243366087</x:v>
       </x:c>
       <x:c r="G17" s="17" t="n">
         <x:f>D17-3.182446305284263*F17</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>-0.10935872046472705</x:v>
       </x:c>
       <x:c r="H17" s="17" t="n">
         <x:f>D17+3.182446305284263*F17</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I17" s="18" t="n">
+        <x:v>1.609358720464727</x:v>
+      </x:c>
+      <x:c r="I17" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!K$4:K$7)+VAR.S('Transformed Scores'!N$4:N$7)+VAR.S('Transformed Scores'!T$4:T$7)+VAR.S('Transformed Scores'!V$4:V$7))/VAR.S('Respondent Scale Means'!G7:J7))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.2857142857142856</x:v>
+      </x:c>
+      <x:c r="J17" s="18" t="n">
+        <x:f>MAX(0,$B$7-D17)</x:f>
+        <x:v>0.73</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -726,27 +757,31 @@
       </x:c>
       <x:c r="D18" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C8:F8)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="E18" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C8:F8)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.5400617248673217</x:v>
       </x:c>
       <x:c r="F18" s="17" t="n">
         <x:f>E18/SQRT(C18)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.27003086243366087</x:v>
       </x:c>
       <x:c r="G18" s="17" t="n">
         <x:f>D18-3.182446305284263*F18</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>0.39064127953527295</x:v>
       </x:c>
       <x:c r="H18" s="17" t="n">
         <x:f>D18+3.182446305284263*F18</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I18" s="18" t="n">
+        <x:v>2.1093587204647273</x:v>
+      </x:c>
+      <x:c r="I18" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!H$4:H$7)+VAR.S('Transformed Scores'!I$4:I$7)+VAR.S('Transformed Scores'!J$4:J$7)+VAR.S('Transformed Scores'!U$4:U$7))/VAR.S('Respondent Scale Means'!G8:J8))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.2857142857142856</x:v>
+      </x:c>
+      <x:c r="J18" s="18" t="n">
+        <x:f>MAX(0,$B$8-D18)</x:f>
+        <x:v>0.10000000000000009</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -766,23 +801,27 @@
       </x:c>
       <x:c r="E19" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C9:F9)</x:f>
-        <x:v>1.1547005383792515</x:v>
+        <x:v>0.408248290463863</x:v>
       </x:c>
       <x:c r="F19" s="17" t="n">
         <x:f>E19/SQRT(C19)</x:f>
-        <x:v>0.5773502691896257</x:v>
+        <x:v>0.2041241452319315</x:v>
       </x:c>
       <x:c r="G19" s="17" t="n">
         <x:f>D19-3.182446305284263*F19</x:f>
-        <x:v>-0.837386231037399</x:v>
+        <x:v>0.3503858681873313</x:v>
       </x:c>
       <x:c r="H19" s="17" t="n">
         <x:f>D19+3.182446305284263*F19</x:f>
-        <x:v>2.837386231037399</x:v>
-      </x:c>
-      <x:c r="I19" s="18" t="n">
+        <x:v>1.6496141318126687</x:v>
+      </x:c>
+      <x:c r="I19" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!F$4:F$7)+VAR.S('Transformed Scores'!M$4:M$7)+VAR.S('Transformed Scores'!R$4:R$7)+VAR.S('Transformed Scores'!AC$4:AC$7))/VAR.S('Respondent Scale Means'!G9:J9))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="J19" s="18" t="n">
+        <x:f>MAX(0,$B$9-D19)</x:f>
+        <x:v>0.1200000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -798,27 +837,31 @@
       </x:c>
       <x:c r="D20" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C10:F10)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="E20" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C10:F10)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.9077852576871218</x:v>
       </x:c>
       <x:c r="F20" s="17" t="n">
         <x:f>E20/SQRT(C20)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.4538926288435609</x:v>
       </x:c>
       <x:c r="G20" s="17" t="n">
         <x:f>D20-3.182446305284263*F20</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-1.1944889196589517</x:v>
       </x:c>
       <x:c r="H20" s="17" t="n">
         <x:f>D20+3.182446305284263*F20</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I20" s="18" t="n">
+        <x:v>1.6944889196589517</x:v>
+      </x:c>
+      <x:c r="I20" s="17" t="n">
         <x:f>(6/(6-1))*(1-(VAR.S('Transformed Scores'!D$9:D$12)+VAR.S('Transformed Scores'!O$9:O$12)+VAR.S('Transformed Scores'!Q$9:Q$12)+VAR.S('Transformed Scores'!S$9:S$12)+VAR.S('Transformed Scores'!AA$9:AA$12)+VAR.S('Transformed Scores'!AB$9:AB$12))/VAR.S('Respondent Scale Means'!G10:J10))</x:f>
-        <x:v>1</x:v>
+        <x:v>0.7887640449438202</x:v>
+      </x:c>
+      <x:c r="J20" s="18" t="n">
+        <x:f>MAX(0,$B$4-D20)</x:f>
+        <x:v>1.33</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -834,27 +877,31 @@
       </x:c>
       <x:c r="D21" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C11:F11)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E21" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C11:F11)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.5400617248673217</x:v>
       </x:c>
       <x:c r="F21" s="17" t="n">
         <x:f>E21/SQRT(C21)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.27003086243366087</x:v>
       </x:c>
       <x:c r="G21" s="17" t="n">
         <x:f>D21-3.182446305284263*F21</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-0.10935872046472705</x:v>
       </x:c>
       <x:c r="H21" s="17" t="n">
         <x:f>D21+3.182446305284263*F21</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I21" s="18" t="n">
+        <x:v>1.609358720464727</x:v>
+      </x:c>
+      <x:c r="I21" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!E$9:E$12)+VAR.S('Transformed Scores'!G$9:G$12)+VAR.S('Transformed Scores'!P$9:P$12)+VAR.S('Transformed Scores'!X$9:X$12))/VAR.S('Respondent Scale Means'!G11:J11))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.2857142857142856</x:v>
+      </x:c>
+      <x:c r="J21" s="18" t="n">
+        <x:f>MAX(0,$B$5-D21)</x:f>
+        <x:v>0.98</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -874,22 +921,26 @@
       </x:c>
       <x:c r="E22" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C12:F12)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.7359800721939872</x:v>
       </x:c>
       <x:c r="F22" s="17" t="n">
         <x:f>E22/SQRT(C22)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.3679900360969936</x:v>
       </x:c>
       <x:c r="G22" s="17" t="n">
         <x:f>D22-3.182446305284263*F22</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-0.6711085307582998</x:v>
       </x:c>
       <x:c r="H22" s="17" t="n">
         <x:f>D22+3.182446305284263*F22</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I22" s="18" t="n">
+        <x:v>1.6711085307582998</x:v>
+      </x:c>
+      <x:c r="I22" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!L$9:L$12)+VAR.S('Transformed Scores'!W$9:W$12)+VAR.S('Transformed Scores'!Y$9:Y$12)+VAR.S('Transformed Scores'!Z$9:Z$12))/VAR.S('Respondent Scale Means'!G12:J12))</x:f>
+        <x:v>0.30769230769230776</x:v>
+      </x:c>
+      <x:c r="J22" s="18" t="n">
+        <x:f>MAX(0,$B$6-D22)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -906,27 +957,31 @@
       </x:c>
       <x:c r="D23" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C13:F13)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="E23" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C13:F13)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.9574271077563381</x:v>
       </x:c>
       <x:c r="F23" s="17" t="n">
         <x:f>E23/SQRT(C23)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.47871355387816905</x:v>
       </x:c>
       <x:c r="G23" s="17" t="n">
         <x:f>D23-3.182446305284263*F23</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-1.273480180829078</x:v>
       </x:c>
       <x:c r="H23" s="17" t="n">
         <x:f>D23+3.182446305284263*F23</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I23" s="18" t="n">
+        <x:v>1.773480180829078</x:v>
+      </x:c>
+      <x:c r="I23" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!K$9:K$12)+VAR.S('Transformed Scores'!N$9:N$12)+VAR.S('Transformed Scores'!T$9:T$12)+VAR.S('Transformed Scores'!V$9:V$12))/VAR.S('Respondent Scale Means'!G13:J13))</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6363636363636362</x:v>
+      </x:c>
+      <x:c r="J23" s="18" t="n">
+        <x:f>MAX(0,$B$7-D23)</x:f>
+        <x:v>1.23</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -942,27 +997,31 @@
       </x:c>
       <x:c r="D24" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C14:F14)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E24" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C14:F14)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.5400617248673217</x:v>
       </x:c>
       <x:c r="F24" s="17" t="n">
         <x:f>E24/SQRT(C24)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.27003086243366087</x:v>
       </x:c>
       <x:c r="G24" s="17" t="n">
         <x:f>D24-3.182446305284263*F24</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-0.10935872046472705</x:v>
       </x:c>
       <x:c r="H24" s="17" t="n">
         <x:f>D24+3.182446305284263*F24</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I24" s="18" t="n">
+        <x:v>1.609358720464727</x:v>
+      </x:c>
+      <x:c r="I24" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!H$9:H$12)+VAR.S('Transformed Scores'!I$9:I$12)+VAR.S('Transformed Scores'!J$9:J$12)+VAR.S('Transformed Scores'!U$9:U$12))/VAR.S('Respondent Scale Means'!G14:J14))</x:f>
-        <x:v>1</x:v>
+        <x:v>-0.2857142857142856</x:v>
+      </x:c>
+      <x:c r="J24" s="18" t="n">
+        <x:f>MAX(0,$B$8-D24)</x:f>
+        <x:v>0.6000000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -982,28 +1041,32 @@
       </x:c>
       <x:c r="E25" s="19" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C15:F15)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.7359800721939872</x:v>
       </x:c>
       <x:c r="F25" s="19" t="n">
         <x:f>E25/SQRT(C25)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.3679900360969936</x:v>
       </x:c>
       <x:c r="G25" s="19" t="n">
         <x:f>D25-3.182446305284263*F25</x:f>
-        <x:v>-1.0912231526421314</x:v>
+        <x:v>-0.6711085307582998</x:v>
       </x:c>
       <x:c r="H25" s="19" t="n">
         <x:f>D25+3.182446305284263*F25</x:f>
-        <x:v>2.091223152642131</x:v>
-      </x:c>
-      <x:c r="I25" s="20" t="n">
+        <x:v>1.6711085307582998</x:v>
+      </x:c>
+      <x:c r="I25" s="19" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!F$9:F$12)+VAR.S('Transformed Scores'!M$9:M$12)+VAR.S('Transformed Scores'!R$9:R$12)+VAR.S('Transformed Scores'!AC$9:AC$12))/VAR.S('Respondent Scale Means'!G15:J15))</x:f>
-        <x:v>1</x:v>
+        <x:v>0.30769230769230776</x:v>
+      </x:c>
+      <x:c r="J25" s="20" t="n">
+        <x:f>MAX(0,$B$9-D25)</x:f>
+        <x:v>0.6200000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22" t="str">
-        <x:v>Expected alpha: 1.000000 for every scale; identical item score vectors give perfect internal consistency.</x:v>
+        <x:v>Cronbach alpha reflects the heterogeneous fixture responses; Gap to Good is formula-derived from the matching threshold and UEQ mean.</x:v>
       </x:c>
       <x:c r="B27" s="22"/>
       <x:c r="C27" s="22"/>
@@ -1013,10 +1076,11 @@
       <x:c r="G27" s="22"/>
       <x:c r="H27" s="22"/>
       <x:c r="I27" s="22"/>
+      <x:c r="J27" s="22"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1677,31 +1741,31 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="12" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="J4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M4" s="12" t="n">
         <x:v>2</x:v>
@@ -1713,46 +1777,46 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="P4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="U4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W4" s="12" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="X4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y4" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA4" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AB4" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC4" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1766,43 +1830,43 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="K5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="n">
         <x:v>6</x:v>
@@ -1811,7 +1875,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="S5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T5" s="12" t="n">
         <x:v>2</x:v>
@@ -1820,10 +1884,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="V5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X5" s="12" t="n">
         <x:v>2</x:v>
@@ -1832,16 +1896,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="Z5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB5" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC5" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1855,7 +1919,7 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:v>4</x:v>
@@ -1864,73 +1928,73 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H6" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="I6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L6" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q6" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="R6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T6" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="U6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="V6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Y6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AA6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AB6" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AC6" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1953,13 +2017,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="I7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J7" s="12" t="n">
         <x:v>4</x:v>
@@ -1971,10 +2035,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="M7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O7" s="12" t="n">
         <x:v>4</x:v>
@@ -1989,37 +2053,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T7" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="U7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y7" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AB7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC7" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2122,31 +2186,31 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I9" s="12" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="J9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M9" s="12" t="n">
         <x:v>2</x:v>
@@ -2158,46 +2222,46 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="P9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="U9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W9" s="12" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="X9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y9" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA9" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AB9" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC9" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2211,76 +2275,76 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="G10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L10" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="N10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="P10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="Q10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S10" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="T10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="U10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V10" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="W10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="X10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z10" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AA10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB10" s="12" t="n">
         <x:v>4</x:v>
@@ -2300,46 +2364,46 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="O11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R11" s="12" t="n">
         <x:v>4</x:v>
@@ -2348,34 +2412,34 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="T11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="W11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA11" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC11" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2398,13 +2462,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H12" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="I12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J12" s="12" t="n">
         <x:v>4</x:v>
@@ -2416,10 +2480,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="M12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O12" s="12" t="n">
         <x:v>4</x:v>
@@ -2434,37 +2498,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T12" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="U12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA12" s="12" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC12" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2733,15 +2797,15 @@
       </x:c>
       <x:c r="D4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D4-4,4-'Raw Answers'!D4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E4-4,4-'Raw Answers'!E4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F4-4,4-'Raw Answers'!F4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G4-4,4-'Raw Answers'!G4)</x:f>
@@ -2749,7 +2813,7 @@
       </x:c>
       <x:c r="H4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H4-4,4-'Raw Answers'!H4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I4-4,4-'Raw Answers'!I4)</x:f>
@@ -2757,15 +2821,15 @@
       </x:c>
       <x:c r="J4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J4-4,4-'Raw Answers'!J4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K4-4,4-'Raw Answers'!K4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L4-4,4-'Raw Answers'!L4)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M4-4,4-'Raw Answers'!M4)</x:f>
@@ -2781,31 +2845,31 @@
       </x:c>
       <x:c r="P4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P4-4,4-'Raw Answers'!P4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q4-4,4-'Raw Answers'!Q4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R4-4,4-'Raw Answers'!R4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S4-4,4-'Raw Answers'!S4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="T4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T4-4,4-'Raw Answers'!T4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U4-4,4-'Raw Answers'!U4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="V4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V4-4,4-'Raw Answers'!V4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="W4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W4-4,4-'Raw Answers'!W4)</x:f>
@@ -2813,15 +2877,15 @@
       </x:c>
       <x:c r="X4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X4-4,4-'Raw Answers'!X4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Y4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y4-4,4-'Raw Answers'!Y4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z4-4,4-'Raw Answers'!Z4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AA4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA4-4,4-'Raw Answers'!AA4)</x:f>
@@ -2829,11 +2893,11 @@
       </x:c>
       <x:c r="AB4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB4-4,4-'Raw Answers'!AB4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC4" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC4-4,4-'Raw Answers'!AC4)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2848,7 +2912,7 @@
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D5-4,4-'Raw Answers'!D5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E5-4,4-'Raw Answers'!E5)</x:f>
@@ -2856,11 +2920,11 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F5-4,4-'Raw Answers'!F5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G5-4,4-'Raw Answers'!G5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H5-4,4-'Raw Answers'!H5)</x:f>
@@ -2868,35 +2932,35 @@
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I5-4,4-'Raw Answers'!I5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J5-4,4-'Raw Answers'!J5)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K5-4,4-'Raw Answers'!K5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L5-4,4-'Raw Answers'!L5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M5-4,4-'Raw Answers'!M5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N5-4,4-'Raw Answers'!N5)</x:f>
-        <x:v>2</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="O5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O5-4,4-'Raw Answers'!O5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P5-4,4-'Raw Answers'!P5)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q5-4,4-'Raw Answers'!Q5)</x:f>
@@ -2908,7 +2972,7 @@
       </x:c>
       <x:c r="S5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S5-4,4-'Raw Answers'!S5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T5-4,4-'Raw Answers'!T5)</x:f>
@@ -2920,11 +2984,11 @@
       </x:c>
       <x:c r="V5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V5-4,4-'Raw Answers'!V5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W5-4,4-'Raw Answers'!W5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="X5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X5-4,4-'Raw Answers'!X5)</x:f>
@@ -2936,19 +3000,19 @@
       </x:c>
       <x:c r="Z5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z5-4,4-'Raw Answers'!Z5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA5-4,4-'Raw Answers'!AA5)</x:f>
-        <x:v>2</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="AB5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB5-4,4-'Raw Answers'!AB5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC5" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC5-4,4-'Raw Answers'!AC5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2963,7 +3027,7 @@
       </x:c>
       <x:c r="D6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D6-4,4-'Raw Answers'!D6)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E6-4,4-'Raw Answers'!E6)</x:f>
@@ -2975,7 +3039,7 @@
       </x:c>
       <x:c r="G6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G6-4,4-'Raw Answers'!G6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H6-4,4-'Raw Answers'!H6)</x:f>
@@ -2983,15 +3047,15 @@
       </x:c>
       <x:c r="I6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I6-4,4-'Raw Answers'!I6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J6-4,4-'Raw Answers'!J6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K6-4,4-'Raw Answers'!K6)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="L6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L6-4,4-'Raw Answers'!L6)</x:f>
@@ -2999,19 +3063,19 @@
       </x:c>
       <x:c r="M6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M6-4,4-'Raw Answers'!M6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N6-4,4-'Raw Answers'!N6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O6-4,4-'Raw Answers'!O6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P6-4,4-'Raw Answers'!P6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q6-4,4-'Raw Answers'!Q6)</x:f>
@@ -3019,11 +3083,11 @@
       </x:c>
       <x:c r="R6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R6-4,4-'Raw Answers'!R6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S6-4,4-'Raw Answers'!S6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T6-4,4-'Raw Answers'!T6)</x:f>
@@ -3031,31 +3095,31 @@
       </x:c>
       <x:c r="U6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U6-4,4-'Raw Answers'!U6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="V6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V6-4,4-'Raw Answers'!V6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W6-4,4-'Raw Answers'!W6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="X6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X6-4,4-'Raw Answers'!X6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Y6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y6-4,4-'Raw Answers'!Y6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z6-4,4-'Raw Answers'!Z6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AA6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA6-4,4-'Raw Answers'!AA6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB6-4,4-'Raw Answers'!AB6)</x:f>
@@ -3063,7 +3127,7 @@
       </x:c>
       <x:c r="AC6" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC6-4,4-'Raw Answers'!AC6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3090,7 +3154,7 @@
       </x:c>
       <x:c r="G7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G7-4,4-'Raw Answers'!G7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H7-4,4-'Raw Answers'!H7)</x:f>
@@ -3098,7 +3162,7 @@
       </x:c>
       <x:c r="I7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I7-4,4-'Raw Answers'!I7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J7-4,4-'Raw Answers'!J7)</x:f>
@@ -3114,11 +3178,11 @@
       </x:c>
       <x:c r="M7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M7-4,4-'Raw Answers'!M7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N7-4,4-'Raw Answers'!N7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O7-4,4-'Raw Answers'!O7)</x:f>
@@ -3138,7 +3202,7 @@
       </x:c>
       <x:c r="S7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S7-4,4-'Raw Answers'!S7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T7-4,4-'Raw Answers'!T7)</x:f>
@@ -3146,19 +3210,19 @@
       </x:c>
       <x:c r="U7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U7-4,4-'Raw Answers'!U7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="V7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V7-4,4-'Raw Answers'!V7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W7-4,4-'Raw Answers'!W7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="X7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X7-4,4-'Raw Answers'!X7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y7-4,4-'Raw Answers'!Y7)</x:f>
@@ -3166,19 +3230,19 @@
       </x:c>
       <x:c r="Z7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z7-4,4-'Raw Answers'!Z7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA7-4,4-'Raw Answers'!AA7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB7-4,4-'Raw Answers'!AB7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC7" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC7-4,4-'Raw Answers'!AC7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3308,15 +3372,15 @@
       </x:c>
       <x:c r="D9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D9-4,4-'Raw Answers'!D9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E9-4,4-'Raw Answers'!E9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F9-4,4-'Raw Answers'!F9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G9-4,4-'Raw Answers'!G9)</x:f>
@@ -3324,7 +3388,7 @@
       </x:c>
       <x:c r="H9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H9-4,4-'Raw Answers'!H9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I9-4,4-'Raw Answers'!I9)</x:f>
@@ -3332,15 +3396,15 @@
       </x:c>
       <x:c r="J9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J9-4,4-'Raw Answers'!J9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K9-4,4-'Raw Answers'!K9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L9-4,4-'Raw Answers'!L9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M9-4,4-'Raw Answers'!M9)</x:f>
@@ -3356,31 +3420,31 @@
       </x:c>
       <x:c r="P9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P9-4,4-'Raw Answers'!P9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q9-4,4-'Raw Answers'!Q9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R9-4,4-'Raw Answers'!R9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S9-4,4-'Raw Answers'!S9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="T9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T9-4,4-'Raw Answers'!T9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U9-4,4-'Raw Answers'!U9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="V9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V9-4,4-'Raw Answers'!V9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="W9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W9-4,4-'Raw Answers'!W9)</x:f>
@@ -3388,15 +3452,15 @@
       </x:c>
       <x:c r="X9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X9-4,4-'Raw Answers'!X9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Y9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y9-4,4-'Raw Answers'!Y9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z9-4,4-'Raw Answers'!Z9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AA9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA9-4,4-'Raw Answers'!AA9)</x:f>
@@ -3404,11 +3468,11 @@
       </x:c>
       <x:c r="AB9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB9-4,4-'Raw Answers'!AB9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC9" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC9-4,4-'Raw Answers'!AC9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3423,11 +3487,11 @@
       </x:c>
       <x:c r="D10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D10-4,4-'Raw Answers'!D10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E10-4,4-'Raw Answers'!E10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F10-4,4-'Raw Answers'!F10)</x:f>
@@ -3435,23 +3499,23 @@
       </x:c>
       <x:c r="G10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G10-4,4-'Raw Answers'!G10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="H10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H10-4,4-'Raw Answers'!H10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I10-4,4-'Raw Answers'!I10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="J10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J10-4,4-'Raw Answers'!J10)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K10-4,4-'Raw Answers'!K10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="L10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L10-4,4-'Raw Answers'!L10)</x:f>
@@ -3459,27 +3523,27 @@
       </x:c>
       <x:c r="M10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M10-4,4-'Raw Answers'!M10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="N10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N10-4,4-'Raw Answers'!N10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="O10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O10-4,4-'Raw Answers'!O10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="P10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P10-4,4-'Raw Answers'!P10)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Q10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q10-4,4-'Raw Answers'!Q10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R10-4,4-'Raw Answers'!R10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S10-4,4-'Raw Answers'!S10)</x:f>
@@ -3487,11 +3551,11 @@
       </x:c>
       <x:c r="T10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T10-4,4-'Raw Answers'!T10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U10-4,4-'Raw Answers'!U10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="V10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V10-4,4-'Raw Answers'!V10)</x:f>
@@ -3499,15 +3563,15 @@
       </x:c>
       <x:c r="W10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W10-4,4-'Raw Answers'!W10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="X10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X10-4,4-'Raw Answers'!X10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y10-4,4-'Raw Answers'!Y10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z10-4,4-'Raw Answers'!Z10)</x:f>
@@ -3515,7 +3579,7 @@
       </x:c>
       <x:c r="AA10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA10-4,4-'Raw Answers'!AA10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="AB10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB10-4,4-'Raw Answers'!AB10)</x:f>
@@ -3538,27 +3602,27 @@
       </x:c>
       <x:c r="D11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D11-4,4-'Raw Answers'!D11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E11-4,4-'Raw Answers'!E11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="F11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F11-4,4-'Raw Answers'!F11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="G11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G11-4,4-'Raw Answers'!G11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H11-4,4-'Raw Answers'!H11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="I11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I11-4,4-'Raw Answers'!I11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J11-4,4-'Raw Answers'!J11)</x:f>
@@ -3566,15 +3630,15 @@
       </x:c>
       <x:c r="K11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K11-4,4-'Raw Answers'!K11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="L11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L11-4,4-'Raw Answers'!L11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="M11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M11-4,4-'Raw Answers'!M11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N11-4,4-'Raw Answers'!N11)</x:f>
@@ -3582,7 +3646,7 @@
       </x:c>
       <x:c r="O11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O11-4,4-'Raw Answers'!O11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P11-4,4-'Raw Answers'!P11)</x:f>
@@ -3590,7 +3654,7 @@
       </x:c>
       <x:c r="Q11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q11-4,4-'Raw Answers'!Q11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="R11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R11-4,4-'Raw Answers'!R11)</x:f>
@@ -3602,11 +3666,11 @@
       </x:c>
       <x:c r="T11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T11-4,4-'Raw Answers'!T11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="U11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U11-4,4-'Raw Answers'!U11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="V11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V11-4,4-'Raw Answers'!V11)</x:f>
@@ -3614,11 +3678,11 @@
       </x:c>
       <x:c r="W11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W11-4,4-'Raw Answers'!W11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="X11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X11-4,4-'Raw Answers'!X11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y11-4,4-'Raw Answers'!Y11)</x:f>
@@ -3626,7 +3690,7 @@
       </x:c>
       <x:c r="Z11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z11-4,4-'Raw Answers'!Z11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA11-4,4-'Raw Answers'!AA11)</x:f>
@@ -3634,11 +3698,11 @@
       </x:c>
       <x:c r="AB11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB11-4,4-'Raw Answers'!AB11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="AC11" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC11-4,4-'Raw Answers'!AC11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3665,7 +3729,7 @@
       </x:c>
       <x:c r="G12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$7="right",'Raw Answers'!G12-4,4-'Raw Answers'!G12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$8="right",'Raw Answers'!H12-4,4-'Raw Answers'!H12)</x:f>
@@ -3673,7 +3737,7 @@
       </x:c>
       <x:c r="I12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$9="right",'Raw Answers'!I12-4,4-'Raw Answers'!I12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$10="right",'Raw Answers'!J12-4,4-'Raw Answers'!J12)</x:f>
@@ -3689,11 +3753,11 @@
       </x:c>
       <x:c r="M12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M12-4,4-'Raw Answers'!M12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N12-4,4-'Raw Answers'!N12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O12-4,4-'Raw Answers'!O12)</x:f>
@@ -3713,7 +3777,7 @@
       </x:c>
       <x:c r="S12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S12-4,4-'Raw Answers'!S12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T12-4,4-'Raw Answers'!T12)</x:f>
@@ -3721,19 +3785,19 @@
       </x:c>
       <x:c r="U12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$21="right",'Raw Answers'!U12-4,4-'Raw Answers'!U12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="V12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$22="right",'Raw Answers'!V12-4,4-'Raw Answers'!V12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$23="right",'Raw Answers'!W12-4,4-'Raw Answers'!W12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="X12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X12-4,4-'Raw Answers'!X12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y12-4,4-'Raw Answers'!Y12)</x:f>
@@ -3741,7 +3805,7 @@
       </x:c>
       <x:c r="Z12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z12-4,4-'Raw Answers'!Z12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA12-4,4-'Raw Answers'!AA12)</x:f>
@@ -3749,11 +3813,11 @@
       </x:c>
       <x:c r="AB12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB12-4,4-'Raw Answers'!AB12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC12" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC12-4,4-'Raw Answers'!AC12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3950,35 +4014,35 @@
       </x:c>
       <x:c r="C4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D4,'Transformed Scores'!O4,'Transformed Scores'!Q4,'Transformed Scores'!S4,'Transformed Scores'!AA4,'Transformed Scores'!AB4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D5,'Transformed Scores'!O5,'Transformed Scores'!Q5,'Transformed Scores'!S5,'Transformed Scores'!AA5,'Transformed Scores'!AB5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="E4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D6,'Transformed Scores'!O6,'Transformed Scores'!Q6,'Transformed Scores'!S6,'Transformed Scores'!AA6,'Transformed Scores'!AB6)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="F4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D7,'Transformed Scores'!O7,'Transformed Scores'!Q7,'Transformed Scores'!S7,'Transformed Scores'!AA7,'Transformed Scores'!AB7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D4,'Transformed Scores'!O4,'Transformed Scores'!Q4,'Transformed Scores'!S4,'Transformed Scores'!AA4,'Transformed Scores'!AB4)</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D5,'Transformed Scores'!O5,'Transformed Scores'!Q5,'Transformed Scores'!S5,'Transformed Scores'!AA5,'Transformed Scores'!AB5)</x:f>
-        <x:v>12</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D6,'Transformed Scores'!O6,'Transformed Scores'!Q6,'Transformed Scores'!S6,'Transformed Scores'!AA6,'Transformed Scores'!AB6)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J4" s="18" t="n">
         <x:f>SUM('Transformed Scores'!D7,'Transformed Scores'!O7,'Transformed Scores'!Q7,'Transformed Scores'!S7,'Transformed Scores'!AA7,'Transformed Scores'!AB7)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3990,35 +4054,35 @@
       </x:c>
       <x:c r="C5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E4,'Transformed Scores'!G4,'Transformed Scores'!P4,'Transformed Scores'!X4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E5,'Transformed Scores'!G5,'Transformed Scores'!P5,'Transformed Scores'!X5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="E5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E6,'Transformed Scores'!G6,'Transformed Scores'!P6,'Transformed Scores'!X6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="F5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E7,'Transformed Scores'!G7,'Transformed Scores'!P7,'Transformed Scores'!X7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E4,'Transformed Scores'!G4,'Transformed Scores'!P4,'Transformed Scores'!X4)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E5,'Transformed Scores'!G5,'Transformed Scores'!P5,'Transformed Scores'!X5)</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E6,'Transformed Scores'!G6,'Transformed Scores'!P6,'Transformed Scores'!X6)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J5" s="18" t="n">
         <x:f>SUM('Transformed Scores'!E7,'Transformed Scores'!G7,'Transformed Scores'!P7,'Transformed Scores'!X7)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4030,35 +4094,35 @@
       </x:c>
       <x:c r="C6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L4,'Transformed Scores'!W4,'Transformed Scores'!Y4,'Transformed Scores'!Z4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L5,'Transformed Scores'!W5,'Transformed Scores'!Y5,'Transformed Scores'!Z5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L6,'Transformed Scores'!W6,'Transformed Scores'!Y6,'Transformed Scores'!Z6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L7,'Transformed Scores'!W7,'Transformed Scores'!Y7,'Transformed Scores'!Z7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L4,'Transformed Scores'!W4,'Transformed Scores'!Y4,'Transformed Scores'!Z4)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L5,'Transformed Scores'!W5,'Transformed Scores'!Y5,'Transformed Scores'!Z5)</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L6,'Transformed Scores'!W6,'Transformed Scores'!Y6,'Transformed Scores'!Z6)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J6" s="18" t="n">
         <x:f>SUM('Transformed Scores'!L7,'Transformed Scores'!W7,'Transformed Scores'!Y7,'Transformed Scores'!Z7)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4070,35 +4134,35 @@
       </x:c>
       <x:c r="C7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K4,'Transformed Scores'!N4,'Transformed Scores'!T4,'Transformed Scores'!V4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K5,'Transformed Scores'!N5,'Transformed Scores'!T5,'Transformed Scores'!V5)</x:f>
-        <x:v>2</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K6,'Transformed Scores'!N6,'Transformed Scores'!T6,'Transformed Scores'!V6)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K7,'Transformed Scores'!N7,'Transformed Scores'!T7,'Transformed Scores'!V7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G7" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K4,'Transformed Scores'!N4,'Transformed Scores'!T4,'Transformed Scores'!V4)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H7" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K5,'Transformed Scores'!N5,'Transformed Scores'!T5,'Transformed Scores'!V5)</x:f>
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I7" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K6,'Transformed Scores'!N6,'Transformed Scores'!T6,'Transformed Scores'!V6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="18" t="n">
         <x:f>SUM('Transformed Scores'!K7,'Transformed Scores'!N7,'Transformed Scores'!T7,'Transformed Scores'!V7)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4110,35 +4174,35 @@
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H4,'Transformed Scores'!I4,'Transformed Scores'!J4,'Transformed Scores'!U4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D8" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H5,'Transformed Scores'!I5,'Transformed Scores'!J5,'Transformed Scores'!U5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="E8" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H6,'Transformed Scores'!I6,'Transformed Scores'!J6,'Transformed Scores'!U6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H7,'Transformed Scores'!I7,'Transformed Scores'!J7,'Transformed Scores'!U7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G8" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H4,'Transformed Scores'!I4,'Transformed Scores'!J4,'Transformed Scores'!U4)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H8" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H5,'Transformed Scores'!I5,'Transformed Scores'!J5,'Transformed Scores'!U5)</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I8" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H6,'Transformed Scores'!I6,'Transformed Scores'!J6,'Transformed Scores'!U6)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J8" s="18" t="n">
         <x:f>SUM('Transformed Scores'!H7,'Transformed Scores'!I7,'Transformed Scores'!J7,'Transformed Scores'!U7)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4150,35 +4214,35 @@
       </x:c>
       <x:c r="C9" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!F4,'Transformed Scores'!M4,'Transformed Scores'!R4,'Transformed Scores'!AC4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D9" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!F5,'Transformed Scores'!M5,'Transformed Scores'!R5,'Transformed Scores'!AC5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!F6,'Transformed Scores'!M6,'Transformed Scores'!R6,'Transformed Scores'!AC6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!F7,'Transformed Scores'!M7,'Transformed Scores'!R7,'Transformed Scores'!AC7)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G9" s="17" t="n">
         <x:f>SUM('Transformed Scores'!F4,'Transformed Scores'!M4,'Transformed Scores'!R4,'Transformed Scores'!AC4)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H9" s="17" t="n">
         <x:f>SUM('Transformed Scores'!F5,'Transformed Scores'!M5,'Transformed Scores'!R5,'Transformed Scores'!AC5)</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I9" s="17" t="n">
         <x:f>SUM('Transformed Scores'!F6,'Transformed Scores'!M6,'Transformed Scores'!R6,'Transformed Scores'!AC6)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J9" s="18" t="n">
         <x:f>SUM('Transformed Scores'!F7,'Transformed Scores'!M7,'Transformed Scores'!R7,'Transformed Scores'!AC7)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4190,35 +4254,35 @@
       </x:c>
       <x:c r="C10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D9,'Transformed Scores'!O9,'Transformed Scores'!Q9,'Transformed Scores'!S9,'Transformed Scores'!AA9,'Transformed Scores'!AB9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D10,'Transformed Scores'!O10,'Transformed Scores'!Q10,'Transformed Scores'!S10,'Transformed Scores'!AA10,'Transformed Scores'!AB10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.5</x:v>
       </x:c>
       <x:c r="E10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D11,'Transformed Scores'!O11,'Transformed Scores'!Q11,'Transformed Scores'!S11,'Transformed Scores'!AA11,'Transformed Scores'!AB11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.3333333333333333</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D12,'Transformed Scores'!O12,'Transformed Scores'!Q12,'Transformed Scores'!S12,'Transformed Scores'!AA12,'Transformed Scores'!AB12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="G10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D9,'Transformed Scores'!O9,'Transformed Scores'!Q9,'Transformed Scores'!S9,'Transformed Scores'!AA9,'Transformed Scores'!AB9)</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D10,'Transformed Scores'!O10,'Transformed Scores'!Q10,'Transformed Scores'!S10,'Transformed Scores'!AA10,'Transformed Scores'!AB10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-3</x:v>
       </x:c>
       <x:c r="I10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D11,'Transformed Scores'!O11,'Transformed Scores'!Q11,'Transformed Scores'!S11,'Transformed Scores'!AA11,'Transformed Scores'!AB11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="J10" s="18" t="n">
         <x:f>SUM('Transformed Scores'!D12,'Transformed Scores'!O12,'Transformed Scores'!Q12,'Transformed Scores'!S12,'Transformed Scores'!AA12,'Transformed Scores'!AB12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4230,35 +4294,35 @@
       </x:c>
       <x:c r="C11" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E9,'Transformed Scores'!G9,'Transformed Scores'!P9,'Transformed Scores'!X9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D11" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E10,'Transformed Scores'!G10,'Transformed Scores'!P10,'Transformed Scores'!X10)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E11" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E11,'Transformed Scores'!G11,'Transformed Scores'!P11,'Transformed Scores'!X11)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E12,'Transformed Scores'!G12,'Transformed Scores'!P12,'Transformed Scores'!X12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E9,'Transformed Scores'!G9,'Transformed Scores'!P9,'Transformed Scores'!X9)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H11" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E10,'Transformed Scores'!G10,'Transformed Scores'!P10,'Transformed Scores'!X10)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I11" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E11,'Transformed Scores'!G11,'Transformed Scores'!P11,'Transformed Scores'!X11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="18" t="n">
         <x:f>SUM('Transformed Scores'!E12,'Transformed Scores'!G12,'Transformed Scores'!P12,'Transformed Scores'!X12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4270,35 +4334,35 @@
       </x:c>
       <x:c r="C12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L9,'Transformed Scores'!W9,'Transformed Scores'!Y9,'Transformed Scores'!Z9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L10,'Transformed Scores'!W10,'Transformed Scores'!Y10,'Transformed Scores'!Z10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.25</x:v>
       </x:c>
       <x:c r="E12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L11,'Transformed Scores'!W11,'Transformed Scores'!Y11,'Transformed Scores'!Z11)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L12,'Transformed Scores'!W12,'Transformed Scores'!Y12,'Transformed Scores'!Z12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G12" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L9,'Transformed Scores'!W9,'Transformed Scores'!Y9,'Transformed Scores'!Z9)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H12" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L10,'Transformed Scores'!W10,'Transformed Scores'!Y10,'Transformed Scores'!Z10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="I12" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L11,'Transformed Scores'!W11,'Transformed Scores'!Y11,'Transformed Scores'!Z11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J12" s="18" t="n">
         <x:f>SUM('Transformed Scores'!L12,'Transformed Scores'!W12,'Transformed Scores'!Y12,'Transformed Scores'!Z12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4310,35 +4374,35 @@
       </x:c>
       <x:c r="C13" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K9,'Transformed Scores'!N9,'Transformed Scores'!T9,'Transformed Scores'!V9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D13" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K10,'Transformed Scores'!N10,'Transformed Scores'!T10,'Transformed Scores'!V10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.5</x:v>
       </x:c>
       <x:c r="E13" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K11,'Transformed Scores'!N11,'Transformed Scores'!T11,'Transformed Scores'!V11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.5</x:v>
       </x:c>
       <x:c r="F13" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K12,'Transformed Scores'!N12,'Transformed Scores'!T12,'Transformed Scores'!V12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G13" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K9,'Transformed Scores'!N9,'Transformed Scores'!T9,'Transformed Scores'!V9)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H13" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K10,'Transformed Scores'!N10,'Transformed Scores'!T10,'Transformed Scores'!V10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="I13" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K11,'Transformed Scores'!N11,'Transformed Scores'!T11,'Transformed Scores'!V11)</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="J13" s="18" t="n">
         <x:f>SUM('Transformed Scores'!K12,'Transformed Scores'!N12,'Transformed Scores'!T12,'Transformed Scores'!V12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4350,35 +4414,35 @@
       </x:c>
       <x:c r="C14" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H9,'Transformed Scores'!I9,'Transformed Scores'!J9,'Transformed Scores'!U9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D14" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H10,'Transformed Scores'!I10,'Transformed Scores'!J10,'Transformed Scores'!U10)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E14" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H11,'Transformed Scores'!I11,'Transformed Scores'!J11,'Transformed Scores'!U11)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!H12,'Transformed Scores'!I12,'Transformed Scores'!J12,'Transformed Scores'!U12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H9,'Transformed Scores'!I9,'Transformed Scores'!J9,'Transformed Scores'!U9)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H14" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H10,'Transformed Scores'!I10,'Transformed Scores'!J10,'Transformed Scores'!U10)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I14" s="17" t="n">
         <x:f>SUM('Transformed Scores'!H11,'Transformed Scores'!I11,'Transformed Scores'!J11,'Transformed Scores'!U11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J14" s="18" t="n">
         <x:f>SUM('Transformed Scores'!H12,'Transformed Scores'!I12,'Transformed Scores'!J12,'Transformed Scores'!U12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4390,35 +4454,35 @@
       </x:c>
       <x:c r="C15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F9,'Transformed Scores'!M9,'Transformed Scores'!R9,'Transformed Scores'!AC9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="D15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F10,'Transformed Scores'!M10,'Transformed Scores'!R10,'Transformed Scores'!AC10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-0.25</x:v>
       </x:c>
       <x:c r="E15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F11,'Transformed Scores'!M11,'Transformed Scores'!R11,'Transformed Scores'!AC11)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F12,'Transformed Scores'!M12,'Transformed Scores'!R12,'Transformed Scores'!AC12)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G15" s="19" t="n">
         <x:f>SUM('Transformed Scores'!F9,'Transformed Scores'!M9,'Transformed Scores'!R9,'Transformed Scores'!AC9)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H15" s="19" t="n">
         <x:f>SUM('Transformed Scores'!F10,'Transformed Scores'!M10,'Transformed Scores'!R10,'Transformed Scores'!AC10)</x:f>
-        <x:v>0</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="I15" s="19" t="n">
         <x:f>SUM('Transformed Scores'!F11,'Transformed Scores'!M11,'Transformed Scores'!R11,'Transformed Scores'!AC11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="20" t="n">
         <x:f>SUM('Transformed Scores'!F12,'Transformed Scores'!M12,'Transformed Scores'!R12,'Transformed Scores'!AC12)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4781,17 +4845,20 @@
         <x:v>ibadah-yu</x:v>
       </x:c>
       <x:c r="B15" s="17" t="n">
+        <x:f>AVERAGE('Overview'!$J$14:$J$19)</x:f>
         <x:v>0.46</x:v>
       </x:c>
       <x:c r="C15" s="17" t="n">
+        <x:f>AVERAGEIF($E$4:$E$9,A15,$F$4:$F$9)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D15" s="17" t="n">
+        <x:f>AVERAGEIF($E$4:$E$9,A15,$G$4:$G$9)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E15" s="17" t="n">
         <x:f>B15/MAX($B$15:$B$16)</x:f>
-        <x:v>0.4791666666666667</x:v>
+        <x:v>0.47916666666666663</x:v>
       </x:c>
       <x:c r="F15" s="17" t="n">
         <x:f>MIN($C$15:$C$16)/C15</x:f>
@@ -4803,7 +4870,7 @@
       </x:c>
       <x:c r="H15" s="17" t="n">
         <x:f>$B$12*E15</x:f>
-        <x:v>0.115</x:v>
+        <x:v>0.11499999999999999</x:v>
       </x:c>
       <x:c r="I15" s="17" t="n">
         <x:f>$C$12*F15</x:f>
@@ -4815,7 +4882,7 @@
       </x:c>
       <x:c r="K15" s="18" t="n">
         <x:f>SUM(H15:J15)</x:f>
-        <x:v>0.7616666666666667</x:v>
+        <x:v>0.7616666666666665</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4823,12 +4890,15 @@
         <x:v>info-yu</x:v>
       </x:c>
       <x:c r="B16" s="17" t="n">
-        <x:v>0.96</x:v>
+        <x:f>AVERAGE('Overview'!$J$20:$J$25)</x:f>
+        <x:v>0.9600000000000001</x:v>
       </x:c>
       <x:c r="C16" s="17" t="n">
+        <x:f>AVERAGEIF($E$4:$E$9,A16,$F$4:$F$9)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D16" s="17" t="n">
+        <x:f>AVERAGEIF($E$4:$E$9,A16,$G$4:$G$9)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E16" s="17" t="n">

</xml_diff>

<commit_message>
fix: distinguish every UEQ golden scale
</commit_message>
<xml_diff>
--- a/docs/research/ueq-saw-golden-fixture.xlsx
+++ b/docs/research/ueq-saw-golden-fixture.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd468ca3291f7411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Mapping" sheetId="2" r:id="R1aade2b990974955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Answers" sheetId="3" r:id="Re9e1450f95aa43c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformed Scores" sheetId="4" r:id="Rba32031370714ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respondent Scale Means" sheetId="5" r:id="R96dbf4eac15f4c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical and SAW" sheetId="6" r:id="R12621751a14f430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf503729ae9a14171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Mapping" sheetId="2" r:id="Rd71ceef5bc324609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Answers" sheetId="3" r:id="R7d18b6377ae64a67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformed Scores" sheetId="4" r:id="R8f50d154d14149fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respondent Scale Means" sheetId="5" r:id="Rdbad30d07fb84f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical and SAW" sheetId="6" r:id="R21fecfb8a68e438a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -597,31 +597,31 @@
       </x:c>
       <x:c r="D14" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C4:F4)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C4:F4)</x:f>
-        <x:v>0.5181877251716008</x:v>
+        <x:v>0.47140452079103173</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:f>E14/SQRT(C14)</x:f>
-        <x:v>0.2590938625858004</x:v>
+        <x:v>0.23570226039551587</x:v>
       </x:c>
       <x:c r="G14" s="17" t="n">
         <x:f>D14-3.182446305284263*F14</x:f>
-        <x:v>-0.07455230570800908</x:v>
+        <x:v>0.24989021225714125</x:v>
       </x:c>
       <x:c r="H14" s="17" t="n">
         <x:f>D14+3.182446305284263*F14</x:f>
-        <x:v>1.574552305708009</x:v>
+        <x:v>1.7501097877428586</x:v>
       </x:c>
       <x:c r="I14" s="17" t="n">
         <x:f>(6/(6-1))*(1-(VAR.S('Transformed Scores'!D$4:D$7)+VAR.S('Transformed Scores'!O$4:O$7)+VAR.S('Transformed Scores'!Q$4:Q$7)+VAR.S('Transformed Scores'!S$4:S$7)+VAR.S('Transformed Scores'!AA$4:AA$7)+VAR.S('Transformed Scores'!AB$4:AB$7))/VAR.S('Respondent Scale Means'!G4:J4))</x:f>
-        <x:v>0.3517241379310345</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="J14" s="18" t="n">
         <x:f>MAX(0,$B$4-D14)</x:f>
-        <x:v>0.8300000000000001</x:v>
+        <x:v>0.5800000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -637,31 +637,31 @@
       </x:c>
       <x:c r="D15" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C5:F5)</x:f>
-        <x:v>1.25</x:v>
+        <x:v>1.125</x:v>
       </x:c>
       <x:c r="E15" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C5:F5)</x:f>
-        <x:v>0.5400617248673217</x:v>
+        <x:v>0.4330127018922193</x:v>
       </x:c>
       <x:c r="F15" s="17" t="n">
         <x:f>E15/SQRT(C15)</x:f>
-        <x:v>0.27003086243366087</x:v>
+        <x:v>0.21650635094610965</x:v>
       </x:c>
       <x:c r="G15" s="17" t="n">
         <x:f>D15-3.182446305284263*F15</x:f>
-        <x:v>0.39064127953527295</x:v>
+        <x:v>0.43598016336097534</x:v>
       </x:c>
       <x:c r="H15" s="17" t="n">
         <x:f>D15+3.182446305284263*F15</x:f>
-        <x:v>2.1093587204647273</x:v>
+        <x:v>1.8140198366390248</x:v>
       </x:c>
       <x:c r="I15" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!E$4:E$7)+VAR.S('Transformed Scores'!G$4:G$7)+VAR.S('Transformed Scores'!P$4:P$7)+VAR.S('Transformed Scores'!X$4:X$7))/VAR.S('Respondent Scale Means'!G5:J5))</x:f>
-        <x:v>-0.2857142857142856</x:v>
+        <x:v>-0.37037037037037024</x:v>
       </x:c>
       <x:c r="J15" s="18" t="n">
         <x:f>MAX(0,$B$5-D15)</x:f>
-        <x:v>0.48</x:v>
+        <x:v>0.605</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -677,23 +677,23 @@
       </x:c>
       <x:c r="D16" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C6:F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="E16" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C6:F6)</x:f>
-        <x:v>0.408248290463863</x:v>
+        <x:v>0.3227486121839514</x:v>
       </x:c>
       <x:c r="F16" s="17" t="n">
         <x:f>E16/SQRT(C16)</x:f>
-        <x:v>0.2041241452319315</x:v>
+        <x:v>0.1613743060919757</x:v>
       </x:c>
       <x:c r="G16" s="17" t="n">
         <x:f>D16-3.182446305284263*F16</x:f>
-        <x:v>0.3503858681873313</x:v>
+        <x:v>0.36143493580978026</x:v>
       </x:c>
       <x:c r="H16" s="17" t="n">
         <x:f>D16+3.182446305284263*F16</x:f>
-        <x:v>1.6496141318126687</x:v>
+        <x:v>1.3885650641902196</x:v>
       </x:c>
       <x:c r="I16" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!L$4:L$7)+VAR.S('Transformed Scores'!W$4:W$7)+VAR.S('Transformed Scores'!Y$4:Y$7)+VAR.S('Transformed Scores'!Z$4:Z$7))/VAR.S('Respondent Scale Means'!G6:J6))</x:f>
@@ -701,7 +701,7 @@
       </x:c>
       <x:c r="J16" s="18" t="n">
         <x:f>MAX(0,$B$6-D16)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -717,31 +717,31 @@
       </x:c>
       <x:c r="D17" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C7:F7)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.6875</x:v>
       </x:c>
       <x:c r="E17" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C7:F7)</x:f>
-        <x:v>0.5400617248673217</x:v>
+        <x:v>0.42695628191498325</x:v>
       </x:c>
       <x:c r="F17" s="17" t="n">
         <x:f>E17/SQRT(C17)</x:f>
-        <x:v>0.27003086243366087</x:v>
+        <x:v>0.21347814095749162</x:v>
       </x:c>
       <x:c r="G17" s="17" t="n">
         <x:f>D17-3.182446305284263*F17</x:f>
-        <x:v>-0.10935872046472705</x:v>
+        <x:v>0.008117279050877668</x:v>
       </x:c>
       <x:c r="H17" s="17" t="n">
         <x:f>D17+3.182446305284263*F17</x:f>
-        <x:v>1.609358720464727</x:v>
+        <x:v>1.3668827209491223</x:v>
       </x:c>
       <x:c r="I17" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!K$4:K$7)+VAR.S('Transformed Scores'!N$4:N$7)+VAR.S('Transformed Scores'!T$4:T$7)+VAR.S('Transformed Scores'!V$4:V$7))/VAR.S('Respondent Scale Means'!G7:J7))</x:f>
-        <x:v>-0.2857142857142856</x:v>
+        <x:v>-0.6857142857142859</x:v>
       </x:c>
       <x:c r="J17" s="18" t="n">
         <x:f>MAX(0,$B$7-D17)</x:f>
-        <x:v>0.73</x:v>
+        <x:v>0.7925</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -797,31 +797,31 @@
       </x:c>
       <x:c r="D19" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C9:F9)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.0625</x:v>
       </x:c>
       <x:c r="E19" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C9:F9)</x:f>
-        <x:v>0.408248290463863</x:v>
+        <x:v>0.3145764348029479</x:v>
       </x:c>
       <x:c r="F19" s="17" t="n">
         <x:f>E19/SQRT(C19)</x:f>
-        <x:v>0.2041241452319315</x:v>
+        <x:v>0.15728821740147395</x:v>
       </x:c>
       <x:c r="G19" s="17" t="n">
         <x:f>D19-3.182446305284263*F19</x:f>
-        <x:v>0.3503858681873313</x:v>
+        <x:v>0.5619386936659313</x:v>
       </x:c>
       <x:c r="H19" s="17" t="n">
         <x:f>D19+3.182446305284263*F19</x:f>
-        <x:v>1.6496141318126687</x:v>
+        <x:v>1.5630613063340686</x:v>
       </x:c>
       <x:c r="I19" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!F$4:F$7)+VAR.S('Transformed Scores'!M$4:M$7)+VAR.S('Transformed Scores'!R$4:R$7)+VAR.S('Transformed Scores'!AC$4:AC$7))/VAR.S('Respondent Scale Means'!G9:J9))</x:f>
-        <x:v>-0.6666666666666666</x:v>
+        <x:v>-2.245614035087719</x:v>
       </x:c>
       <x:c r="J19" s="18" t="n">
         <x:f>MAX(0,$B$9-D19)</x:f>
-        <x:v>0.1200000000000001</x:v>
+        <x:v>0.05750000000000011</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -837,31 +837,31 @@
       </x:c>
       <x:c r="D20" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C10:F10)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.375</x:v>
       </x:c>
       <x:c r="E20" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C10:F10)</x:f>
-        <x:v>0.9077852576871218</x:v>
+        <x:v>0.8319432851039965</x:v>
       </x:c>
       <x:c r="F20" s="17" t="n">
         <x:f>E20/SQRT(C20)</x:f>
-        <x:v>0.4538926288435609</x:v>
+        <x:v>0.41597164255199826</x:v>
       </x:c>
       <x:c r="G20" s="17" t="n">
         <x:f>D20-3.182446305284263*F20</x:f>
-        <x:v>-1.1944889196589517</x:v>
+        <x:v>-0.9488074169426328</x:v>
       </x:c>
       <x:c r="H20" s="17" t="n">
         <x:f>D20+3.182446305284263*F20</x:f>
-        <x:v>1.6944889196589517</x:v>
+        <x:v>1.6988074169426328</x:v>
       </x:c>
       <x:c r="I20" s="17" t="n">
         <x:f>(6/(6-1))*(1-(VAR.S('Transformed Scores'!D$9:D$12)+VAR.S('Transformed Scores'!O$9:O$12)+VAR.S('Transformed Scores'!Q$9:Q$12)+VAR.S('Transformed Scores'!S$9:S$12)+VAR.S('Transformed Scores'!AA$9:AA$12)+VAR.S('Transformed Scores'!AB$9:AB$12))/VAR.S('Respondent Scale Means'!G10:J10))</x:f>
-        <x:v>0.7887640449438202</x:v>
+        <x:v>0.7625418060200669</x:v>
       </x:c>
       <x:c r="J20" s="18" t="n">
         <x:f>MAX(0,$B$4-D20)</x:f>
-        <x:v>1.33</x:v>
+        <x:v>1.205</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -877,31 +877,31 @@
       </x:c>
       <x:c r="D21" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C11:F11)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.6875</x:v>
       </x:c>
       <x:c r="E21" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C11:F11)</x:f>
-        <x:v>0.5400617248673217</x:v>
+        <x:v>0.590726953281576</x:v>
       </x:c>
       <x:c r="F21" s="17" t="n">
         <x:f>E21/SQRT(C21)</x:f>
-        <x:v>0.27003086243366087</x:v>
+        <x:v>0.295363476640788</x:v>
       </x:c>
       <x:c r="G21" s="17" t="n">
         <x:f>D21-3.182446305284263*F21</x:f>
-        <x:v>-0.10935872046472705</x:v>
+        <x:v>-0.2524784049513904</x:v>
       </x:c>
       <x:c r="H21" s="17" t="n">
         <x:f>D21+3.182446305284263*F21</x:f>
-        <x:v>1.609358720464727</x:v>
+        <x:v>1.6274784049513904</x:v>
       </x:c>
       <x:c r="I21" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!E$9:E$12)+VAR.S('Transformed Scores'!G$9:G$12)+VAR.S('Transformed Scores'!P$9:P$12)+VAR.S('Transformed Scores'!X$9:X$12))/VAR.S('Respondent Scale Means'!G11:J11))</x:f>
-        <x:v>-0.2857142857142856</x:v>
+        <x:v>-0.03980099502487573</x:v>
       </x:c>
       <x:c r="J21" s="18" t="n">
         <x:f>MAX(0,$B$5-D21)</x:f>
-        <x:v>0.98</x:v>
+        <x:v>1.0425</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -917,31 +917,31 @@
       </x:c>
       <x:c r="D22" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C12:F12)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.5625</x:v>
       </x:c>
       <x:c r="E22" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C12:F12)</x:f>
-        <x:v>0.7359800721939872</x:v>
+        <x:v>0.6574889099191459</x:v>
       </x:c>
       <x:c r="F22" s="17" t="n">
         <x:f>E22/SQRT(C22)</x:f>
-        <x:v>0.3679900360969936</x:v>
+        <x:v>0.32874445495957294</x:v>
       </x:c>
       <x:c r="G22" s="17" t="n">
         <x:f>D22-3.182446305284263*F22</x:f>
-        <x:v>-0.6711085307582998</x:v>
+        <x:v>-0.48371157606878157</x:v>
       </x:c>
       <x:c r="H22" s="17" t="n">
         <x:f>D22+3.182446305284263*F22</x:f>
-        <x:v>1.6711085307582998</x:v>
+        <x:v>1.6087115760687816</x:v>
       </x:c>
       <x:c r="I22" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!L$9:L$12)+VAR.S('Transformed Scores'!W$9:W$12)+VAR.S('Transformed Scores'!Y$9:Y$12)+VAR.S('Transformed Scores'!Z$9:Z$12))/VAR.S('Respondent Scale Means'!G12:J12))</x:f>
-        <x:v>0.30769230769230776</x:v>
+        <x:v>0.06425702811245015</x:v>
       </x:c>
       <x:c r="J22" s="18" t="n">
         <x:f>MAX(0,$B$6-D22)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.9375</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -957,31 +957,31 @@
       </x:c>
       <x:c r="D23" s="17" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C13:F13)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.1875</x:v>
       </x:c>
       <x:c r="E23" s="17" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C13:F13)</x:f>
-        <x:v>0.9574271077563381</x:v>
+        <x:v>0.9437293044088437</x:v>
       </x:c>
       <x:c r="F23" s="17" t="n">
         <x:f>E23/SQRT(C23)</x:f>
-        <x:v>0.47871355387816905</x:v>
+        <x:v>0.47186465220442186</x:v>
       </x:c>
       <x:c r="G23" s="17" t="n">
         <x:f>D23-3.182446305284263*F23</x:f>
-        <x:v>-1.273480180829078</x:v>
+        <x:v>-1.314183919002206</x:v>
       </x:c>
       <x:c r="H23" s="17" t="n">
         <x:f>D23+3.182446305284263*F23</x:f>
-        <x:v>1.773480180829078</x:v>
+        <x:v>1.689183919002206</x:v>
       </x:c>
       <x:c r="I23" s="17" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!K$9:K$12)+VAR.S('Transformed Scores'!N$9:N$12)+VAR.S('Transformed Scores'!T$9:T$12)+VAR.S('Transformed Scores'!V$9:V$12))/VAR.S('Respondent Scale Means'!G13:J13))</x:f>
-        <x:v>0.6363636363636362</x:v>
+        <x:v>0.6393762183235867</x:v>
       </x:c>
       <x:c r="J23" s="18" t="n">
         <x:f>MAX(0,$B$7-D23)</x:f>
-        <x:v>1.23</x:v>
+        <x:v>1.2925</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1037,31 +1037,31 @@
       </x:c>
       <x:c r="D25" s="19" t="n">
         <x:f>AVERAGE('Respondent Scale Means'!C15:F15)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.4375</x:v>
       </x:c>
       <x:c r="E25" s="19" t="n">
         <x:f>STDEV.S('Respondent Scale Means'!C15:F15)</x:f>
-        <x:v>0.7359800721939872</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="F25" s="19" t="n">
         <x:f>E25/SQRT(C25)</x:f>
-        <x:v>0.3679900360969936</x:v>
+        <x:v>0.3125</x:v>
       </x:c>
       <x:c r="G25" s="19" t="n">
         <x:f>D25-3.182446305284263*F25</x:f>
-        <x:v>-0.6711085307582998</x:v>
+        <x:v>-0.5570144704013321</x:v>
       </x:c>
       <x:c r="H25" s="19" t="n">
         <x:f>D25+3.182446305284263*F25</x:f>
-        <x:v>1.6711085307582998</x:v>
+        <x:v>1.4320144704013322</x:v>
       </x:c>
       <x:c r="I25" s="19" t="n">
         <x:f>(4/(4-1))*(1-(VAR.S('Transformed Scores'!F$9:F$12)+VAR.S('Transformed Scores'!M$9:M$12)+VAR.S('Transformed Scores'!R$9:R$12)+VAR.S('Transformed Scores'!AC$9:AC$12))/VAR.S('Respondent Scale Means'!G15:J15))</x:f>
-        <x:v>0.30769230769230776</x:v>
+        <x:v>-0.07111111111111097</x:v>
       </x:c>
       <x:c r="J25" s="20" t="n">
         <x:f>MAX(0,$B$9-D25)</x:f>
-        <x:v>0.6200000000000001</x:v>
+        <x:v>0.6825000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1744,7 +1744,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
         <x:v>1</x:v>
@@ -1762,10 +1762,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="K4" s="12" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L4" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M4" s="12" t="n">
         <x:v>2</x:v>
@@ -1786,7 +1786,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="S4" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T4" s="12" t="n">
         <x:v>3</x:v>
@@ -1863,10 +1863,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="O5" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P5" s="12" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="n">
         <x:v>6</x:v>
@@ -1893,13 +1893,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Y5" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z5" s="12" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AA5" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB5" s="12" t="n">
         <x:v>3</x:v>
@@ -1919,7 +1919,7 @@
         <x:v>included</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:v>4</x:v>
@@ -1991,7 +1991,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AB6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC6" s="13" t="n">
         <x:v>6</x:v>
@@ -2047,7 +2047,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q7" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R7" s="12" t="n">
         <x:v>4</x:v>
@@ -2083,7 +2083,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AC7" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2228,7 +2228,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="R9" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S9" s="12" t="n">
         <x:v>4</x:v>
@@ -2299,7 +2299,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="L10" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M10" s="12" t="n">
         <x:v>6</x:v>
@@ -2308,7 +2308,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="O10" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P10" s="12" t="n">
         <x:v>6</x:v>
@@ -2409,7 +2409,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S11" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T11" s="12" t="n">
         <x:v>5</x:v>
@@ -2483,7 +2483,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N12" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O12" s="12" t="n">
         <x:v>4</x:v>
@@ -2513,7 +2513,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="X12" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:v>4</x:v>
@@ -2522,7 +2522,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AA12" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AB12" s="12" t="n">
         <x:v>3</x:v>
@@ -2801,7 +2801,7 @@
       </x:c>
       <x:c r="E4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E4-4,4-'Raw Answers'!E4)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$6="right",'Raw Answers'!F4-4,4-'Raw Answers'!F4)</x:f>
@@ -2825,11 +2825,11 @@
       </x:c>
       <x:c r="K4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$11="right",'Raw Answers'!K4-4,4-'Raw Answers'!K4)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L4-4,4-'Raw Answers'!L4)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M4-4,4-'Raw Answers'!M4)</x:f>
@@ -2857,7 +2857,7 @@
       </x:c>
       <x:c r="S4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S4-4,4-'Raw Answers'!S4)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T4" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T4-4,4-'Raw Answers'!T4)</x:f>
@@ -2956,11 +2956,11 @@
       </x:c>
       <x:c r="O5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O5-4,4-'Raw Answers'!O5)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P5-4,4-'Raw Answers'!P5)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q5-4,4-'Raw Answers'!Q5)</x:f>
@@ -2996,7 +2996,7 @@
       </x:c>
       <x:c r="Y5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y5-4,4-'Raw Answers'!Y5)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$26="right",'Raw Answers'!Z5-4,4-'Raw Answers'!Z5)</x:f>
@@ -3004,7 +3004,7 @@
       </x:c>
       <x:c r="AA5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA5-4,4-'Raw Answers'!AA5)</x:f>
-        <x:v>-1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AB5" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB5-4,4-'Raw Answers'!AB5)</x:f>
@@ -3027,7 +3027,7 @@
       </x:c>
       <x:c r="D6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$4="right",'Raw Answers'!D6-4,4-'Raw Answers'!D6)</x:f>
-        <x:v>-1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$5="right",'Raw Answers'!E6-4,4-'Raw Answers'!E6)</x:f>
@@ -3123,7 +3123,7 @@
       </x:c>
       <x:c r="AB6" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB6-4,4-'Raw Answers'!AB6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC6" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC6-4,4-'Raw Answers'!AC6)</x:f>
@@ -3194,7 +3194,7 @@
       </x:c>
       <x:c r="Q7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$17="right",'Raw Answers'!Q7-4,4-'Raw Answers'!Q7)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R7" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R7-4,4-'Raw Answers'!R7)</x:f>
@@ -3242,7 +3242,7 @@
       </x:c>
       <x:c r="AC7" s="13" t="n">
         <x:f>IF('Item Mapping'!$E$29="right",'Raw Answers'!AC7-4,4-'Raw Answers'!AC7)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3428,7 +3428,7 @@
       </x:c>
       <x:c r="R9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$18="right",'Raw Answers'!R9-4,4-'Raw Answers'!R9)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S9" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S9-4,4-'Raw Answers'!S9)</x:f>
@@ -3519,7 +3519,7 @@
       </x:c>
       <x:c r="L10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$12="right",'Raw Answers'!L10-4,4-'Raw Answers'!L10)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$13="right",'Raw Answers'!M10-4,4-'Raw Answers'!M10)</x:f>
@@ -3531,7 +3531,7 @@
       </x:c>
       <x:c r="O10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O10-4,4-'Raw Answers'!O10)</x:f>
-        <x:v>-2</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="P10" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$16="right",'Raw Answers'!P10-4,4-'Raw Answers'!P10)</x:f>
@@ -3662,7 +3662,7 @@
       </x:c>
       <x:c r="S11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$19="right",'Raw Answers'!S11-4,4-'Raw Answers'!S11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T11" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$20="right",'Raw Answers'!T11-4,4-'Raw Answers'!T11)</x:f>
@@ -3757,7 +3757,7 @@
       </x:c>
       <x:c r="N12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$14="right",'Raw Answers'!N12-4,4-'Raw Answers'!N12)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$15="right",'Raw Answers'!O12-4,4-'Raw Answers'!O12)</x:f>
@@ -3797,7 +3797,7 @@
       </x:c>
       <x:c r="X12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$24="right",'Raw Answers'!X12-4,4-'Raw Answers'!X12)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$25="right",'Raw Answers'!Y12-4,4-'Raw Answers'!Y12)</x:f>
@@ -3809,7 +3809,7 @@
       </x:c>
       <x:c r="AA12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$27="right",'Raw Answers'!AA12-4,4-'Raw Answers'!AA12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB12" s="12" t="n">
         <x:f>IF('Item Mapping'!$E$28="right",'Raw Answers'!AB12-4,4-'Raw Answers'!AB12)</x:f>
@@ -4014,35 +4014,35 @@
       </x:c>
       <x:c r="C4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D4,'Transformed Scores'!O4,'Transformed Scores'!Q4,'Transformed Scores'!S4,'Transformed Scores'!AA4,'Transformed Scores'!AB4)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.6666666666666667</x:v>
       </x:c>
       <x:c r="D4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D5,'Transformed Scores'!O5,'Transformed Scores'!Q5,'Transformed Scores'!S5,'Transformed Scores'!AA5,'Transformed Scores'!AB5)</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D6,'Transformed Scores'!O6,'Transformed Scores'!Q6,'Transformed Scores'!S6,'Transformed Scores'!AA6,'Transformed Scores'!AB6)</x:f>
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="F4" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D7,'Transformed Scores'!O7,'Transformed Scores'!Q7,'Transformed Scores'!S7,'Transformed Scores'!AA7,'Transformed Scores'!AB7)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D4,'Transformed Scores'!O4,'Transformed Scores'!Q4,'Transformed Scores'!S4,'Transformed Scores'!AA4,'Transformed Scores'!AB4)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D5,'Transformed Scores'!O5,'Transformed Scores'!Q5,'Transformed Scores'!S5,'Transformed Scores'!AA5,'Transformed Scores'!AB5)</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I4" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D6,'Transformed Scores'!O6,'Transformed Scores'!Q6,'Transformed Scores'!S6,'Transformed Scores'!AA6,'Transformed Scores'!AB6)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J4" s="18" t="n">
         <x:f>SUM('Transformed Scores'!D7,'Transformed Scores'!O7,'Transformed Scores'!Q7,'Transformed Scores'!S7,'Transformed Scores'!AA7,'Transformed Scores'!AB7)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4054,11 +4054,11 @@
       </x:c>
       <x:c r="C5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E4,'Transformed Scores'!G4,'Transformed Scores'!P4,'Transformed Scores'!X4)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="D5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E5,'Transformed Scores'!G5,'Transformed Scores'!P5,'Transformed Scores'!X5)</x:f>
-        <x:v>1.75</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="E5" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E6,'Transformed Scores'!G6,'Transformed Scores'!P6,'Transformed Scores'!X6)</x:f>
@@ -4070,11 +4070,11 @@
       </x:c>
       <x:c r="G5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E4,'Transformed Scores'!G4,'Transformed Scores'!P4,'Transformed Scores'!X4)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E5,'Transformed Scores'!G5,'Transformed Scores'!P5,'Transformed Scores'!X5)</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I5" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E6,'Transformed Scores'!G6,'Transformed Scores'!P6,'Transformed Scores'!X6)</x:f>
@@ -4094,11 +4094,11 @@
       </x:c>
       <x:c r="C6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L4,'Transformed Scores'!W4,'Transformed Scores'!Y4,'Transformed Scores'!Z4)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="D6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L5,'Transformed Scores'!W5,'Transformed Scores'!Y5,'Transformed Scores'!Z5)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="E6" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L6,'Transformed Scores'!W6,'Transformed Scores'!Y6,'Transformed Scores'!Z6)</x:f>
@@ -4110,11 +4110,11 @@
       </x:c>
       <x:c r="G6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L4,'Transformed Scores'!W4,'Transformed Scores'!Y4,'Transformed Scores'!Z4)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L5,'Transformed Scores'!W5,'Transformed Scores'!Y5,'Transformed Scores'!Z5)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I6" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L6,'Transformed Scores'!W6,'Transformed Scores'!Y6,'Transformed Scores'!Z6)</x:f>
@@ -4134,7 +4134,7 @@
       </x:c>
       <x:c r="C7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K4,'Transformed Scores'!N4,'Transformed Scores'!T4,'Transformed Scores'!V4)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="D7" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K5,'Transformed Scores'!N5,'Transformed Scores'!T5,'Transformed Scores'!V5)</x:f>
@@ -4150,7 +4150,7 @@
       </x:c>
       <x:c r="G7" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K4,'Transformed Scores'!N4,'Transformed Scores'!T4,'Transformed Scores'!V4)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H7" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K5,'Transformed Scores'!N5,'Transformed Scores'!T5,'Transformed Scores'!V5)</x:f>
@@ -4226,7 +4226,7 @@
       </x:c>
       <x:c r="F9" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!F7,'Transformed Scores'!M7,'Transformed Scores'!R7,'Transformed Scores'!AC7)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="G9" s="17" t="n">
         <x:f>SUM('Transformed Scores'!F4,'Transformed Scores'!M4,'Transformed Scores'!R4,'Transformed Scores'!AC4)</x:f>
@@ -4242,7 +4242,7 @@
       </x:c>
       <x:c r="J9" s="18" t="n">
         <x:f>SUM('Transformed Scores'!F7,'Transformed Scores'!M7,'Transformed Scores'!R7,'Transformed Scores'!AC7)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4258,15 +4258,15 @@
       </x:c>
       <x:c r="D10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D10,'Transformed Scores'!O10,'Transformed Scores'!Q10,'Transformed Scores'!S10,'Transformed Scores'!AA10,'Transformed Scores'!AB10)</x:f>
-        <x:v>-0.5</x:v>
+        <x:v>-0.3333333333333333</x:v>
       </x:c>
       <x:c r="E10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D11,'Transformed Scores'!O11,'Transformed Scores'!Q11,'Transformed Scores'!S11,'Transformed Scores'!AA11,'Transformed Scores'!AB11)</x:f>
-        <x:v>-0.3333333333333333</x:v>
+        <x:v>-0.16666666666666666</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!D12,'Transformed Scores'!O12,'Transformed Scores'!Q12,'Transformed Scores'!S12,'Transformed Scores'!AA12,'Transformed Scores'!AB12)</x:f>
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D9,'Transformed Scores'!O9,'Transformed Scores'!Q9,'Transformed Scores'!S9,'Transformed Scores'!AA9,'Transformed Scores'!AB9)</x:f>
@@ -4274,15 +4274,15 @@
       </x:c>
       <x:c r="H10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D10,'Transformed Scores'!O10,'Transformed Scores'!Q10,'Transformed Scores'!S10,'Transformed Scores'!AA10,'Transformed Scores'!AB10)</x:f>
-        <x:v>-3</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="I10" s="17" t="n">
         <x:f>SUM('Transformed Scores'!D11,'Transformed Scores'!O11,'Transformed Scores'!Q11,'Transformed Scores'!S11,'Transformed Scores'!AA11,'Transformed Scores'!AB11)</x:f>
-        <x:v>-2</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="J10" s="18" t="n">
         <x:f>SUM('Transformed Scores'!D12,'Transformed Scores'!O12,'Transformed Scores'!Q12,'Transformed Scores'!S12,'Transformed Scores'!AA12,'Transformed Scores'!AB12)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4306,7 +4306,7 @@
       </x:c>
       <x:c r="F11" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!E12,'Transformed Scores'!G12,'Transformed Scores'!P12,'Transformed Scores'!X12)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
         <x:f>SUM('Transformed Scores'!E9,'Transformed Scores'!G9,'Transformed Scores'!P9,'Transformed Scores'!X9)</x:f>
@@ -4322,7 +4322,7 @@
       </x:c>
       <x:c r="J11" s="18" t="n">
         <x:f>SUM('Transformed Scores'!E12,'Transformed Scores'!G12,'Transformed Scores'!P12,'Transformed Scores'!X12)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4338,7 +4338,7 @@
       </x:c>
       <x:c r="D12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L10,'Transformed Scores'!W10,'Transformed Scores'!Y10,'Transformed Scores'!Z10)</x:f>
-        <x:v>-0.25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!L11,'Transformed Scores'!W11,'Transformed Scores'!Y11,'Transformed Scores'!Z11)</x:f>
@@ -4354,7 +4354,7 @@
       </x:c>
       <x:c r="H12" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L10,'Transformed Scores'!W10,'Transformed Scores'!Y10,'Transformed Scores'!Z10)</x:f>
-        <x:v>-1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="17" t="n">
         <x:f>SUM('Transformed Scores'!L11,'Transformed Scores'!W11,'Transformed Scores'!Y11,'Transformed Scores'!Z11)</x:f>
@@ -4386,7 +4386,7 @@
       </x:c>
       <x:c r="F13" s="17" t="n">
         <x:f>AVERAGE('Transformed Scores'!K12,'Transformed Scores'!N12,'Transformed Scores'!T12,'Transformed Scores'!V12)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="G13" s="17" t="n">
         <x:f>SUM('Transformed Scores'!K9,'Transformed Scores'!N9,'Transformed Scores'!T9,'Transformed Scores'!V9)</x:f>
@@ -4402,7 +4402,7 @@
       </x:c>
       <x:c r="J13" s="18" t="n">
         <x:f>SUM('Transformed Scores'!K12,'Transformed Scores'!N12,'Transformed Scores'!T12,'Transformed Scores'!V12)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4454,7 +4454,7 @@
       </x:c>
       <x:c r="C15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F9,'Transformed Scores'!M9,'Transformed Scores'!R9,'Transformed Scores'!AC9)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="D15" s="19" t="n">
         <x:f>AVERAGE('Transformed Scores'!F10,'Transformed Scores'!M10,'Transformed Scores'!R10,'Transformed Scores'!AC10)</x:f>
@@ -4470,7 +4470,7 @@
       </x:c>
       <x:c r="G15" s="19" t="n">
         <x:f>SUM('Transformed Scores'!F9,'Transformed Scores'!M9,'Transformed Scores'!R9,'Transformed Scores'!AC9)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H15" s="19" t="n">
         <x:f>SUM('Transformed Scores'!F10,'Transformed Scores'!M10,'Transformed Scores'!R10,'Transformed Scores'!AC10)</x:f>

</xml_diff>